<commit_message>
Artefatos Validados / Publisher 2.3.4
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-BRTipoDocumento.xlsx
+++ b/docs/CodeSystem-BRTipoDocumento.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="62">
   <si>
     <t>Property</t>
   </si>
@@ -199,18 +199,6 @@
   </si>
   <si>
     <t>Atestado Médico/Odontológico</t>
-  </si>
-  <si>
-    <t>REPM</t>
-  </si>
-  <si>
-    <t>Registro Eletrônico da Prescrição de Medicamento</t>
-  </si>
-  <si>
-    <t>REDFM</t>
-  </si>
-  <si>
-    <t>Registro Eletrônico de Dispensação ou Fornecimento de Medicamentos</t>
   </si>
 </sst>
 </file>
@@ -518,7 +506,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -649,30 +637,6 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11">
-      <c r="A11" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="B11" t="s" s="2">
-        <v>62</v>
-      </c>
-      <c r="C11" t="s" s="2">
-        <v>63</v>
-      </c>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="B12" t="s" s="2">
-        <v>64</v>
-      </c>
-      <c r="C12" t="s" s="2">
-        <v>65</v>
-      </c>
-      <c r="D12" s="2"/>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>